<commit_message>
Rev. C 2K: yeni ETNA 26, vitrin 3×6, 17 BLADE 12, hareketli sunum + ayrıntı sayfası
</commit_message>
<xml_diff>
--- a/Malzeme_Listesi.xlsx
+++ b/Malzeme_Listesi.xlsx
@@ -542,13 +542,13 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>50</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1721</v>
+        <v>2021</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>447</v>
+        <v>525</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2014</v>
+        <v>2365</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>24163</v>
+        <v>28375</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>

</xml_diff>